<commit_message>
attach mclust per call, it was masking purrr::map for everything downstream
</commit_message>
<xml_diff>
--- a/03_Features/03_Subtypes/c_data/01_subtypes.xlsx
+++ b/03_Features/03_Subtypes/c_data/01_subtypes.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">space</t>
   </si>
@@ -75,6 +75,15 @@
     <t xml:space="preserve">fcsa_II</t>
   </si>
   <si>
+    <t xml:space="preserve">fcsa_mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nfibre_mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nfibre_I</t>
+  </si>
+  <si>
     <t xml:space="preserve">mcsa</t>
   </si>
   <si>
@@ -82,6 +91,9 @@
   </si>
   <si>
     <t xml:space="preserve">1rm_ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">volume_load</t>
   </si>
 </sst>
 </file>
@@ -735,7 +747,7 @@
         <v>15</v>
       </c>
       <c r="D6" t="n">
-        <v>0.050632911392405</v>
+        <v>-0.0253164556962026</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -752,10 +764,10 @@
         <v>22</v>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0762732319575188</v>
+        <v>-0.0632911392405064</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -766,16 +778,16 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C8" t="n">
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0305343511450382</v>
+        <v>-0.0632911392405064</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -786,16 +798,16 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C9" t="n">
         <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0687022900763359</v>
+        <v>0.050632911392405</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -806,16 +818,16 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0687022900763359</v>
+        <v>-0.0762732319575188</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -826,16 +838,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C11" t="n">
         <v>15</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0305343511450382</v>
+        <v>-0.0632911392405064</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -849,13 +861,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C12" t="n">
         <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.16030534351145</v>
+        <v>-0.0305343511450382</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -869,18 +881,178 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E16" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C17" t="n">
+        <v>15</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.0305343511450382</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.16030534351145</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" t="n">
         <v>14</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D20" t="n">
         <v>-0.0581395348837209</v>
       </c>
-      <c r="E13" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="n">
+        <v>15</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.0687022900763359</v>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>